<commit_message>
Actualización completa informe Puebla y correcciones finales
</commit_message>
<xml_diff>
--- a/data/DatosActividad_TablaMortalidadGuatemala2018.xlsx
+++ b/data/DatosActividad_TablaMortalidadGuatemala2018.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\angel\Documents\DEMOGRAFÍA\DEMOGRAPHY_9219\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5465D02-455A-4CE8-BCA9-29E512BBDF5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C429A2D-CE0E-40F9-BEF8-AF58801AC0D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{AA1FD95C-5C7D-4022-A558-3323BFE15373}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{AA1FD95C-5C7D-4022-A558-3323BFE15373}"/>
   </bookViews>
   <sheets>
     <sheet name="tabla mortalidad 1998" sheetId="2" r:id="rId1"/>
@@ -19,7 +19,7 @@
   <definedNames>
     <definedName name="_Hlk25056703" localSheetId="1">'tabla mortalidad 2018'!$A$3</definedName>
   </definedNames>
-  <calcPr calcId="191028" iterate="1" iterateCount="1000" calcOnSave="0"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -540,11 +540,11 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -27914,7 +27914,7 @@
       <c r="S21" s="1"/>
     </row>
     <row r="22" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A22" s="22" t="s">
+      <c r="A22" s="21" t="s">
         <v>13</v>
       </c>
       <c r="B22" s="12"/>
@@ -28690,7 +28690,7 @@
         <v>2439804.7273956439</v>
       </c>
       <c r="M16" s="13">
-        <f t="shared" si="5"/>
+        <f>L16/I16</f>
         <v>27.649406433438916</v>
       </c>
       <c r="O16" s="1"/>
@@ -29002,12 +29002,12 @@
       <c r="O22" s="1"/>
     </row>
     <row r="48" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C48" s="21" t="s">
+      <c r="C48" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="D48" s="21"/>
-      <c r="E48" s="21"/>
-      <c r="F48" s="21"/>
+      <c r="D48" s="22"/>
+      <c r="E48" s="22"/>
+      <c r="F48" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>